<commit_message>
Update import cost 2026-06-18 (CPO696-3 송금, CPO696-5/MPO67-68/APO001/GPO475 신규)
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260618.xlsx
+++ b/RNR_수입원가_2026_20260618.xlsx
@@ -2206,12 +2206,12 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE5" s="3" t="inlineStr">
+      <c r="AE5" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF5" s="4" t="inlineStr">
+      <c r="AF5" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2333,12 +2333,12 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE6" s="3" t="inlineStr">
+      <c r="AE6" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF6" s="4" t="inlineStr">
+      <c r="AF6" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2460,12 +2460,12 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE7" s="3" t="inlineStr">
+      <c r="AE7" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF7" s="4" t="inlineStr">
+      <c r="AF7" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2587,12 +2587,12 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="AE8" s="3" t="inlineStr">
+      <c r="AE8" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF8" s="4" t="inlineStr">
+      <c r="AF8" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2657,7 +2657,7 @@
           <t>Parts (국내)</t>
         </is>
       </c>
-      <c r="O9" s="12" t="n"/>
+      <c r="O9" s="177" t="n"/>
       <c r="P9" s="12" t="n"/>
       <c r="Q9" s="18">
         <f>IF(P9="","",IFERROR(VLOOKUP(O9,FxRateTable,4,TRUE),""))</f>
@@ -2673,7 +2673,7 @@
       <c r="T9" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="U9" s="13" t="n">
+      <c r="U9" s="176" t="n">
         <v>0</v>
       </c>
       <c r="V9" s="12" t="inlineStr">
@@ -2708,12 +2708,12 @@
         <v/>
       </c>
       <c r="AD9" s="12" t="n"/>
-      <c r="AE9" s="12" t="inlineStr">
+      <c r="AE9" s="177" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF9" s="13" t="inlineStr">
+      <c r="AF9" s="176" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2835,12 +2835,12 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE10" s="3" t="inlineStr">
+      <c r="AE10" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF10" s="4" t="inlineStr">
+      <c r="AF10" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2962,12 +2962,12 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE11" s="3" t="inlineStr">
+      <c r="AE11" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF11" s="4" t="inlineStr">
+      <c r="AF11" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3089,12 +3089,12 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE12" s="3" t="inlineStr">
+      <c r="AE12" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF12" s="4" t="inlineStr">
+      <c r="AF12" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3216,12 +3216,12 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE13" s="3" t="inlineStr">
+      <c r="AE13" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF13" s="4" t="inlineStr">
+      <c r="AF13" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3343,12 +3343,12 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE14" s="3" t="inlineStr">
+      <c r="AE14" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF14" s="4" t="inlineStr">
+      <c r="AF14" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3470,12 +3470,12 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="AE15" s="3" t="inlineStr">
+      <c r="AE15" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF15" s="4" t="inlineStr">
+      <c r="AF15" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3597,12 +3597,12 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="AE16" s="3" t="inlineStr">
+      <c r="AE16" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF16" s="4" t="inlineStr">
+      <c r="AF16" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3724,12 +3724,12 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="AE17" s="3" t="inlineStr">
+      <c r="AE17" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF17" s="4" t="inlineStr">
+      <c r="AF17" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3851,12 +3851,12 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE18" s="3" t="inlineStr">
+      <c r="AE18" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF18" s="4" t="inlineStr">
+      <c r="AF18" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3978,12 +3978,12 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="AE19" s="3" t="inlineStr">
+      <c r="AE19" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF19" s="4" t="inlineStr">
+      <c r="AF19" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4105,12 +4105,12 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="AE20" s="3" t="inlineStr">
+      <c r="AE20" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF20" s="4" t="inlineStr">
+      <c r="AF20" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4232,12 +4232,12 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="AE21" s="3" t="inlineStr">
+      <c r="AE21" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF21" s="4" t="inlineStr">
+      <c r="AF21" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4359,12 +4359,12 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="AE22" s="3" t="inlineStr">
+      <c r="AE22" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF22" s="4" t="inlineStr">
+      <c r="AF22" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4429,7 +4429,7 @@
           <t>Projector (한국)</t>
         </is>
       </c>
-      <c r="O23" s="12" t="n"/>
+      <c r="O23" s="177" t="n"/>
       <c r="P23" s="12" t="n"/>
       <c r="Q23" s="18">
         <f>IF(P23="","",IFERROR(VLOOKUP(O23,FxRateTable,4,TRUE),""))</f>
@@ -4445,7 +4445,7 @@
       <c r="T23" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="U23" s="13" t="n">
+      <c r="U23" s="176" t="n">
         <v>0</v>
       </c>
       <c r="V23" s="12" t="inlineStr">
@@ -4480,12 +4480,12 @@
         <v/>
       </c>
       <c r="AD23" s="12" t="n"/>
-      <c r="AE23" s="12" t="inlineStr">
+      <c r="AE23" s="177" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF23" s="13" t="inlineStr">
+      <c r="AF23" s="176" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4607,12 +4607,12 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE24" s="3" t="inlineStr">
+      <c r="AE24" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF24" s="4" t="inlineStr">
+      <c r="AF24" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4734,12 +4734,12 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE25" s="3" t="inlineStr">
+      <c r="AE25" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF25" s="4" t="inlineStr">
+      <c r="AF25" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4861,12 +4861,12 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE26" s="3" t="inlineStr">
+      <c r="AE26" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF26" s="4" t="inlineStr">
+      <c r="AF26" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4988,12 +4988,12 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE27" s="3" t="inlineStr">
+      <c r="AE27" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF27" s="4" t="inlineStr">
+      <c r="AF27" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5115,12 +5115,12 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE28" s="3" t="inlineStr">
+      <c r="AE28" s="175" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF28" s="4" t="inlineStr">
+      <c r="AF28" s="174" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5238,8 +5238,8 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE29" s="3" t="n"/>
-      <c r="AF29" s="4" t="n"/>
+      <c r="AE29" s="175" t="n"/>
+      <c r="AF29" s="174" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="78" t="n">
@@ -5353,8 +5353,8 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE30" s="78" t="n"/>
-      <c r="AF30" s="78" t="n"/>
+      <c r="AE30" s="179" t="n"/>
+      <c r="AF30" s="179" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="78" t="n">
@@ -5468,8 +5468,8 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE31" s="78" t="n"/>
-      <c r="AF31" s="78" t="n"/>
+      <c r="AE31" s="179" t="n"/>
+      <c r="AF31" s="179" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="78" t="n">
@@ -5573,8 +5573,8 @@
         <v/>
       </c>
       <c r="AD32" s="78" t="n"/>
-      <c r="AE32" s="78" t="n"/>
-      <c r="AF32" s="78" t="n"/>
+      <c r="AE32" s="179" t="n"/>
+      <c r="AF32" s="179" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="124" t="n">
@@ -5603,7 +5603,7 @@
       <c r="F33" s="181" t="n">
         <v>46127</v>
       </c>
-      <c r="G33" s="283" t="n">
+      <c r="G33" s="181" t="n">
         <v>46190</v>
       </c>
       <c r="H33" s="126" t="n">
@@ -5647,7 +5647,7 @@
       <c r="T33" s="128" t="n">
         <v>52140300</v>
       </c>
-      <c r="U33" s="129" t="n"/>
+      <c r="U33" s="182" t="n"/>
       <c r="V33" s="129" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
@@ -5684,8 +5684,8 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE33" s="129" t="n"/>
-      <c r="AF33" s="129" t="n"/>
+      <c r="AE33" s="182" t="n"/>
+      <c r="AF33" s="182" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="124" t="n">
@@ -5714,7 +5714,7 @@
       <c r="F34" s="181" t="n">
         <v>46143</v>
       </c>
-      <c r="G34" s="124" t="inlineStr">
+      <c r="G34" s="181" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5764,7 +5764,7 @@
       <c r="T34" s="128" t="n">
         <v>118665800</v>
       </c>
-      <c r="U34" s="129" t="n"/>
+      <c r="U34" s="182" t="n"/>
       <c r="V34" s="129" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
@@ -5801,8 +5801,8 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE34" s="129" t="n"/>
-      <c r="AF34" s="129" t="n"/>
+      <c r="AE34" s="182" t="n"/>
+      <c r="AF34" s="182" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="124" t="n">
@@ -5875,7 +5875,7 @@
       <c r="T35" s="128" t="n">
         <v>14902330</v>
       </c>
-      <c r="U35" s="129" t="n"/>
+      <c r="U35" s="182" t="n"/>
       <c r="V35" s="129" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
@@ -5912,8 +5912,8 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE35" s="129" t="n"/>
-      <c r="AF35" s="129" t="n"/>
+      <c r="AE35" s="182" t="n"/>
+      <c r="AF35" s="182" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="124" t="n">
@@ -5964,7 +5964,7 @@
         <v>7</v>
       </c>
       <c r="N36" s="129" t="n"/>
-      <c r="O36" s="129" t="n"/>
+      <c r="O36" s="182" t="n"/>
       <c r="P36" s="129" t="n"/>
       <c r="Q36" s="126">
         <f>IF(P36="","",IFERROR(VLOOKUP(O36,FxRateTable,4,TRUE),""))</f>
@@ -5980,7 +5980,7 @@
       <c r="T36" s="128" t="n">
         <v>0</v>
       </c>
-      <c r="U36" s="129" t="n"/>
+      <c r="U36" s="182" t="n"/>
       <c r="V36" s="129" t="n"/>
       <c r="W36" s="128" t="n">
         <v>0</v>
@@ -6009,8 +6009,8 @@
         <v/>
       </c>
       <c r="AD36" s="129" t="n"/>
-      <c r="AE36" s="129" t="n"/>
-      <c r="AF36" s="129" t="n"/>
+      <c r="AE36" s="182" t="n"/>
+      <c r="AF36" s="182" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="207" t="n">
@@ -6124,8 +6124,8 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE37" s="207" t="n"/>
-      <c r="AF37" s="208" t="n"/>
+      <c r="AE37" s="210" t="n"/>
+      <c r="AF37" s="209" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="207" t="n">
@@ -6239,8 +6239,8 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE38" s="207" t="n"/>
-      <c r="AF38" s="208" t="n"/>
+      <c r="AE38" s="210" t="n"/>
+      <c r="AF38" s="209" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="124" t="n">
@@ -6303,7 +6303,7 @@
           <t>JNIOR Model 410 (IPO017, FedEx 4/21 발송분)</t>
         </is>
       </c>
-      <c r="O39" s="129" t="n"/>
+      <c r="O39" s="182" t="n"/>
       <c r="P39" s="129" t="n"/>
       <c r="Q39" s="126">
         <f>IF(P39="","",IFERROR(VLOOKUP(O39,FxRateTable,4,TRUE),""))</f>
@@ -6319,7 +6319,7 @@
       <c r="T39" s="128" t="n">
         <v>0</v>
       </c>
-      <c r="U39" s="129" t="n"/>
+      <c r="U39" s="182" t="n"/>
       <c r="V39" s="129" t="inlineStr">
         <is>
           <t>-</t>
@@ -6352,12 +6352,12 @@
         <v/>
       </c>
       <c r="AD39" s="129" t="n"/>
-      <c r="AE39" s="129" t="inlineStr">
+      <c r="AE39" s="182" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF39" s="129" t="inlineStr">
+      <c r="AF39" s="182" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6390,7 +6390,7 @@
       <c r="F40" s="181" t="n">
         <v>46163</v>
       </c>
-      <c r="G40" s="283" t="inlineStr">
+      <c r="G40" s="181" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6444,7 +6444,7 @@
       <c r="T40" s="128" t="n">
         <v>52536040</v>
       </c>
-      <c r="U40" s="129" t="n"/>
+      <c r="U40" s="182" t="n"/>
       <c r="V40" s="129" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
@@ -6481,8 +6481,8 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="AE40" s="129" t="n"/>
-      <c r="AF40" s="129" t="n"/>
+      <c r="AE40" s="182" t="n"/>
+      <c r="AF40" s="182" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="124" t="n">
@@ -6511,7 +6511,7 @@
       <c r="F41" s="181" t="n">
         <v>46154</v>
       </c>
-      <c r="G41" s="283" t="n">
+      <c r="G41" s="181" t="n">
         <v>46190</v>
       </c>
       <c r="H41" s="126" t="n">
@@ -6559,7 +6559,7 @@
       <c r="T41" s="128" t="n">
         <v>8891915</v>
       </c>
-      <c r="U41" s="129" t="n"/>
+      <c r="U41" s="182" t="n"/>
       <c r="V41" s="129" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
@@ -6596,8 +6596,8 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="AE41" s="129" t="n"/>
-      <c r="AF41" s="129" t="n"/>
+      <c r="AE41" s="182" t="n"/>
+      <c r="AF41" s="182" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="124" t="n">
@@ -6626,7 +6626,7 @@
       <c r="F42" s="181" t="n">
         <v>46154</v>
       </c>
-      <c r="G42" s="283" t="n">
+      <c r="G42" s="181" t="n">
         <v>46190</v>
       </c>
       <c r="H42" s="126" t="n">
@@ -6674,7 +6674,7 @@
       <c r="T42" s="128" t="n">
         <v>2096763</v>
       </c>
-      <c r="U42" s="129" t="n"/>
+      <c r="U42" s="182" t="n"/>
       <c r="V42" s="129" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
@@ -6711,8 +6711,8 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="AE42" s="129" t="n"/>
-      <c r="AF42" s="129" t="n"/>
+      <c r="AE42" s="182" t="n"/>
+      <c r="AF42" s="182" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="124" t="n">
@@ -6741,7 +6741,7 @@
       <c r="F43" s="181" t="n">
         <v>46163</v>
       </c>
-      <c r="G43" s="283" t="n">
+      <c r="G43" s="181" t="n">
         <v>46190</v>
       </c>
       <c r="H43" s="126" t="n">
@@ -6783,7 +6783,7 @@
       <c r="T43" s="128" t="n">
         <v>0</v>
       </c>
-      <c r="U43" s="129" t="n"/>
+      <c r="U43" s="182" t="n"/>
       <c r="V43" s="129" t="n"/>
       <c r="W43" s="128" t="n">
         <v>0</v>
@@ -6812,8 +6812,8 @@
         <v/>
       </c>
       <c r="AD43" s="129" t="n"/>
-      <c r="AE43" s="129" t="n"/>
-      <c r="AF43" s="129" t="n"/>
+      <c r="AE43" s="182" t="n"/>
+      <c r="AF43" s="182" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="20" t="n">
@@ -6868,7 +6868,7 @@
           <t>EW CP2220</t>
         </is>
       </c>
-      <c r="O44" s="20" t="inlineStr">
+      <c r="O44" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6892,7 +6892,7 @@
       <c r="T44" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U44" s="21" t="n">
+      <c r="U44" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V44" s="20" t="inlineStr">
@@ -6995,7 +6995,7 @@
           <t>HFR License</t>
         </is>
       </c>
-      <c r="O45" s="20" t="inlineStr">
+      <c r="O45" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7019,7 +7019,7 @@
       <c r="T45" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U45" s="21" t="n">
+      <c r="U45" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V45" s="20" t="inlineStr">
@@ -7122,7 +7122,7 @@
           <t>EW CP2309/2315/2320-RGB</t>
         </is>
       </c>
-      <c r="O46" s="20" t="inlineStr">
+      <c r="O46" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7146,7 +7146,7 @@
       <c r="T46" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U46" s="21" t="n">
+      <c r="U46" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V46" s="20" t="inlineStr">
@@ -7249,7 +7249,7 @@
           <t>TMS-2000 EW</t>
         </is>
       </c>
-      <c r="O47" s="20" t="inlineStr">
+      <c r="O47" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7273,7 +7273,7 @@
       <c r="T47" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U47" s="21" t="n">
+      <c r="U47" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V47" s="20" t="inlineStr">
@@ -7376,7 +7376,7 @@
           <t>TMS-1000 EW</t>
         </is>
       </c>
-      <c r="O48" s="20" t="inlineStr">
+      <c r="O48" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7400,7 +7400,7 @@
       <c r="T48" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U48" s="21" t="n">
+      <c r="U48" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V48" s="20" t="inlineStr">
@@ -7503,7 +7503,7 @@
           <t>EW 대량 (CP2208~CP4450)</t>
         </is>
       </c>
-      <c r="O49" s="20" t="inlineStr">
+      <c r="O49" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7527,7 +7527,7 @@
       <c r="T49" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U49" s="21" t="n">
+      <c r="U49" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V49" s="20" t="inlineStr">
@@ -7636,7 +7636,7 @@
           <t>EW 대량 (SR/SX/TMS)</t>
         </is>
       </c>
-      <c r="O50" s="20" t="inlineStr">
+      <c r="O50" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7660,7 +7660,7 @@
       <c r="T50" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U50" s="21" t="n">
+      <c r="U50" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V50" s="20" t="inlineStr">
@@ -7763,7 +7763,7 @@
           <t>EW CP2315/CP4440-RGB</t>
         </is>
       </c>
-      <c r="O51" s="20" t="inlineStr">
+      <c r="O51" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7787,7 +7787,7 @@
       <c r="T51" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U51" s="21" t="n">
+      <c r="U51" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V51" s="20" t="inlineStr">
@@ -7896,7 +7896,7 @@
           <t>EW (홀딩)</t>
         </is>
       </c>
-      <c r="O52" s="20" t="inlineStr">
+      <c r="O52" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7920,7 +7920,7 @@
       <c r="T52" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U52" s="21" t="n">
+      <c r="U52" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V52" s="20" t="inlineStr">
@@ -8023,7 +8023,7 @@
           <t>TMS-2000 License</t>
         </is>
       </c>
-      <c r="O53" s="20" t="inlineStr">
+      <c r="O53" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8047,7 +8047,7 @@
       <c r="T53" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U53" s="21" t="n">
+      <c r="U53" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V53" s="20" t="inlineStr">
@@ -8150,7 +8150,7 @@
           <t>SX/SR EW (CGV/Lotte)</t>
         </is>
       </c>
-      <c r="O54" s="20" t="inlineStr">
+      <c r="O54" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8174,7 +8174,7 @@
       <c r="T54" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U54" s="21" t="n">
+      <c r="U54" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V54" s="20" t="inlineStr">
@@ -8277,7 +8277,7 @@
           <t>SR-1000/SX-3000 EW</t>
         </is>
       </c>
-      <c r="O55" s="20" t="inlineStr">
+      <c r="O55" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8301,7 +8301,7 @@
       <c r="T55" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U55" s="21" t="n">
+      <c r="U55" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V55" s="20" t="inlineStr">
@@ -8404,7 +8404,7 @@
           <t>EW (메가박스 외)</t>
         </is>
       </c>
-      <c r="O56" s="20" t="inlineStr">
+      <c r="O56" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8428,7 +8428,7 @@
       <c r="T56" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U56" s="21" t="n">
+      <c r="U56" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V56" s="20" t="inlineStr">
@@ -8531,7 +8531,7 @@
           <t>SR/SX EW (하남미사 외)</t>
         </is>
       </c>
-      <c r="O57" s="20" t="inlineStr">
+      <c r="O57" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8555,7 +8555,7 @@
       <c r="T57" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U57" s="21" t="n">
+      <c r="U57" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V57" s="20" t="inlineStr">
@@ -8658,7 +8658,7 @@
           <t>TMS-1000 License</t>
         </is>
       </c>
-      <c r="O58" s="20" t="inlineStr">
+      <c r="O58" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8682,7 +8682,7 @@
       <c r="T58" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U58" s="21" t="n">
+      <c r="U58" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V58" s="20" t="inlineStr">
@@ -8785,7 +8785,7 @@
           <t>Dolby Atmos License</t>
         </is>
       </c>
-      <c r="O59" s="20" t="inlineStr">
+      <c r="O59" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8809,7 +8809,7 @@
       <c r="T59" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U59" s="21" t="n">
+      <c r="U59" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V59" s="20" t="inlineStr">
@@ -8912,7 +8912,7 @@
           <t>EW (CGV 동백 외)</t>
         </is>
       </c>
-      <c r="O60" s="20" t="inlineStr">
+      <c r="O60" s="184" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8936,7 +8936,7 @@
       <c r="T60" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="U60" s="21" t="n">
+      <c r="U60" s="183" t="n">
         <v>0</v>
       </c>
       <c r="V60" s="20" t="inlineStr">
@@ -9283,7 +9283,7 @@
         <v>8000</v>
       </c>
       <c r="N63" s="137" t="n"/>
-      <c r="O63" s="137" t="n"/>
+      <c r="O63" s="189" t="n"/>
       <c r="P63" s="137" t="n"/>
       <c r="Q63" s="134">
         <f>IF(P63="","",IFERROR(VLOOKUP(O63,FxRateTable,4,TRUE),""))</f>
@@ -9299,7 +9299,7 @@
       <c r="T63" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="U63" s="137" t="n"/>
+      <c r="U63" s="189" t="n"/>
       <c r="V63" s="137" t="n"/>
       <c r="W63" s="136" t="n">
         <v>0</v>
@@ -9388,7 +9388,7 @@
         <v>20</v>
       </c>
       <c r="N64" s="137" t="n"/>
-      <c r="O64" s="137" t="n"/>
+      <c r="O64" s="189" t="n"/>
       <c r="P64" s="137" t="n"/>
       <c r="Q64" s="134">
         <f>IF(P64="","",IFERROR(VLOOKUP(O64,FxRateTable,4,TRUE),""))</f>
@@ -9404,7 +9404,7 @@
       <c r="T64" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="U64" s="137" t="n"/>
+      <c r="U64" s="189" t="n"/>
       <c r="V64" s="137" t="n"/>
       <c r="W64" s="136" t="n">
         <v>0</v>
@@ -9471,7 +9471,7 @@
       <c r="F65" s="188" t="n">
         <v>46152</v>
       </c>
-      <c r="G65" s="233" t="n">
+      <c r="G65" s="188" t="n">
         <v>46183</v>
       </c>
       <c r="H65" s="134" t="n">
@@ -9493,7 +9493,7 @@
         <v>34</v>
       </c>
       <c r="N65" s="137" t="n"/>
-      <c r="O65" s="137" t="n"/>
+      <c r="O65" s="189" t="n"/>
       <c r="P65" s="137" t="n"/>
       <c r="Q65" s="134">
         <f>IF(P65="","",IFERROR(VLOOKUP(O65,FxRateTable,4,TRUE),""))</f>
@@ -9509,7 +9509,7 @@
       <c r="T65" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="U65" s="137" t="n"/>
+      <c r="U65" s="189" t="n"/>
       <c r="V65" s="137" t="n"/>
       <c r="W65" s="136" t="n">
         <v>0</v>
@@ -9542,12 +9542,12 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="AE65" s="137" t="inlineStr">
+      <c r="AE65" s="189" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF65" s="137" t="inlineStr">
+      <c r="AF65" s="189" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9606,7 +9606,7 @@
           <t>TMS-1000 License 6 screens (CGV 안동)</t>
         </is>
       </c>
-      <c r="O66" s="137" t="n"/>
+      <c r="O66" s="189" t="n"/>
       <c r="P66" s="137" t="n"/>
       <c r="Q66" s="134">
         <f>IF(P66="","",IFERROR(VLOOKUP(O66,FxRateTable,4,TRUE),""))</f>
@@ -9622,7 +9622,7 @@
       <c r="T66" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="U66" s="137" t="n"/>
+      <c r="U66" s="189" t="n"/>
       <c r="V66" s="137" t="n"/>
       <c r="W66" s="136" t="n">
         <v>0</v>
@@ -9721,7 +9721,7 @@
           <t>Inspection fee</t>
         </is>
       </c>
-      <c r="O67" s="12" t="inlineStr">
+      <c r="O67" s="177" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9745,7 +9745,7 @@
       <c r="T67" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="U67" s="13" t="n">
+      <c r="U67" s="176" t="n">
         <v>0</v>
       </c>
       <c r="V67" s="12" t="inlineStr">
@@ -9874,7 +9874,7 @@
       <c r="T68" s="18" t="n">
         <v>67750</v>
       </c>
-      <c r="U68" s="13" t="n"/>
+      <c r="U68" s="176" t="n"/>
       <c r="V68" s="12" t="inlineStr">
         <is>
           <t>운서합동</t>
@@ -10027,8 +10027,8 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE69" s="216" t="n"/>
-      <c r="AF69" s="217" t="n"/>
+      <c r="AE69" s="219" t="n"/>
+      <c r="AF69" s="218" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="284" t="n">
@@ -10099,7 +10099,7 @@
       <c r="T70" s="290" t="n">
         <v>0</v>
       </c>
-      <c r="U70" s="285" t="n"/>
+      <c r="U70" s="286" t="n"/>
       <c r="V70" s="284" t="n"/>
       <c r="W70" s="290" t="n">
         <v>0</v>
@@ -13494,7 +13494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M98"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12.83203125" customWidth="1" style="160" min="1" max="1"/>
@@ -17916,7 +17916,6 @@
         <v/>
       </c>
     </row>
-    <row r="98"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A41:L41"/>

</xml_diff>